<commit_message>
CI Build: Synchronisation of the project's models with the google sheet metadata version  11079
Add lineage property to taxon
</commit_message>
<xml_diff>
--- a/models/subsidiary_models/excel/evora_schema.xlsx
+++ b/models/subsidiary_models/excel/evora_schema.xlsx
@@ -2146,7 +2146,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R1"/>
+  <dimension ref="A1:S1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2192,50 +2192,55 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>lineage</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>title</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>weight</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>inVocabulary</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>keyword</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>dateIssued</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>dateModified</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>identifier</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>iri</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>publisher</t>
         </is>

</xml_diff>